<commit_message>
back2back inverter simulink model
Ttype modulation SVPWM
</commit_message>
<xml_diff>
--- a/IEMDC-2025/Final Paper Codes/SemiconductorLosses/Semiconductor Losses.xlsx
+++ b/IEMDC-2025/Final Paper Codes/SemiconductorLosses/Semiconductor Losses.xlsx
@@ -19,7 +19,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="51">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="305" uniqueCount="51">
   <si>
     <t>Operating Point</t>
   </si>
@@ -178,7 +178,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
-  <fonts count="8" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -234,6 +234,13 @@
       <b/>
       <sz val="11"/>
       <color rgb="FF7030A0"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -403,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="28">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1"/>
@@ -441,6 +448,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -559,23 +567,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$5:$E$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -583,23 +594,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$5:$F$9</c:f>
+              <c:f>Sheet1!$F$5:$F$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1096</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1449</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1802</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2155</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2508</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2861</c:v>
                 </c:pt>
               </c:numCache>
@@ -632,23 +646,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$5:$E$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -656,23 +673,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$5:$M$9</c:f>
+              <c:f>Sheet1!$M$5:$M$10</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1410</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1574</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1738</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>1900</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2066</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2230</c:v>
                 </c:pt>
               </c:numCache>
@@ -981,23 +1001,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$12:$E$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1005,23 +1028,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$11:$F$15</c:f>
+              <c:f>Sheet1!$F$12:$F$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1156</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1521</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1891</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2256</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2620</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2991</c:v>
                 </c:pt>
               </c:numCache>
@@ -1054,23 +1080,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$12:$E$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1078,23 +1107,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$11:$M$15</c:f>
+              <c:f>Sheet1!$M$12:$M$17</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1263</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1436</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1610</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>1784</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1955</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2132</c:v>
                 </c:pt>
               </c:numCache>
@@ -1403,23 +1435,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$19:$E$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1427,23 +1462,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$17:$F$21</c:f>
+              <c:f>Sheet1!$F$19:$F$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>362</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>527</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>698</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>863</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1028</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1199</c:v>
                 </c:pt>
               </c:numCache>
@@ -1476,23 +1514,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$19:$E$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1500,23 +1541,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$17:$M$21</c:f>
+              <c:f>Sheet1!$M$19:$M$24</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>460</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>540</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>620</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>700</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>777</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>860</c:v>
                 </c:pt>
               </c:numCache>
@@ -1825,23 +1869,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$26:$E$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1849,23 +1896,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$23:$F$27</c:f>
+              <c:f>Sheet1!$F$26:$F$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>159</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>260</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>366</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>467</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>568</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>674</c:v>
                 </c:pt>
               </c:numCache>
@@ -1898,23 +1948,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$26:$E$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -1922,23 +1975,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$23:$M$27</c:f>
+              <c:f>Sheet1!$M$26:$M$31</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>217</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>270</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>323</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>375</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>428</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>481</c:v>
                 </c:pt>
               </c:numCache>
@@ -2247,23 +2303,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$33:$E$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -2271,23 +2330,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$29:$F$33</c:f>
+              <c:f>Sheet1!$F$33:$F$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1093</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1446</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1798</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>2150</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>2501</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2852</c:v>
                 </c:pt>
               </c:numCache>
@@ -2320,23 +2382,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$33:$E$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -2344,23 +2409,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$29:$M$33</c:f>
+              <c:f>Sheet1!$M$33:$M$38</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>1215</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>1384</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>1549</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>1719</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1883</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>2053</c:v>
                 </c:pt>
               </c:numCache>
@@ -2669,23 +2737,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$40:$E$45</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -2693,23 +2764,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$F$35:$F$39</c:f>
+              <c:f>Sheet1!$F$40:$F$45</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>474</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>675</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>870</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>1067</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>1264</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1462</c:v>
                 </c:pt>
               </c:numCache>
@@ -2742,23 +2816,26 @@
           </c:marker>
           <c:cat>
             <c:numRef>
-              <c:f>Sheet1!$E$5:$E$9</c:f>
+              <c:f>Sheet1!$E$40:$E$45</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>5</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>10</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>15</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>20</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>25</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>30</c:v>
                 </c:pt>
               </c:numCache>
@@ -2766,23 +2843,26 @@
           </c:cat>
           <c:val>
             <c:numRef>
-              <c:f>Sheet1!$M$35:$M$39</c:f>
+              <c:f>Sheet1!$M$40:$M$45</c:f>
               <c:numCache>
                 <c:formatCode>General</c:formatCode>
-                <c:ptCount val="5"/>
+                <c:ptCount val="6"/>
                 <c:pt idx="0">
+                  <c:v>572</c:v>
+                </c:pt>
+                <c:pt idx="1">
                   <c:v>659</c:v>
                 </c:pt>
-                <c:pt idx="1">
+                <c:pt idx="2">
                   <c:v>747</c:v>
                 </c:pt>
-                <c:pt idx="2">
+                <c:pt idx="3">
                   <c:v>840</c:v>
                 </c:pt>
-                <c:pt idx="3">
+                <c:pt idx="4">
                   <c:v>927</c:v>
                 </c:pt>
-                <c:pt idx="4">
+                <c:pt idx="5">
                   <c:v>1015</c:v>
                 </c:pt>
               </c:numCache>
@@ -6339,7 +6419,7 @@
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>104775</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6363,13 +6443,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>457200</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>123825</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>152400</xdr:colOff>
-      <xdr:row>33</xdr:row>
+      <xdr:row>38</xdr:row>
       <xdr:rowOff>9525</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6395,13 +6475,13 @@
     <xdr:from>
       <xdr:col>14</xdr:col>
       <xdr:colOff>490818</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>77320</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>22</xdr:col>
       <xdr:colOff>186018</xdr:colOff>
-      <xdr:row>46</xdr:row>
+      <xdr:row>52</xdr:row>
       <xdr:rowOff>145676</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6433,7 +6513,7 @@
     <xdr:to>
       <xdr:col>30</xdr:col>
       <xdr:colOff>81243</xdr:colOff>
-      <xdr:row>17</xdr:row>
+      <xdr:row>20</xdr:row>
       <xdr:rowOff>6164</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6459,13 +6539,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>439270</xdr:colOff>
-      <xdr:row>18</xdr:row>
+      <xdr:row>21</xdr:row>
       <xdr:rowOff>63873</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
       <xdr:colOff>134470</xdr:colOff>
-      <xdr:row>32</xdr:row>
+      <xdr:row>37</xdr:row>
       <xdr:rowOff>141754</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6491,13 +6571,13 @@
     <xdr:from>
       <xdr:col>22</xdr:col>
       <xdr:colOff>513790</xdr:colOff>
-      <xdr:row>34</xdr:row>
+      <xdr:row>40</xdr:row>
       <xdr:rowOff>153521</xdr:rowOff>
     </xdr:from>
     <xdr:to>
       <xdr:col>30</xdr:col>
       <xdr:colOff>213472</xdr:colOff>
-      <xdr:row>47</xdr:row>
+      <xdr:row>53</xdr:row>
       <xdr:rowOff>29696</xdr:rowOff>
     </xdr:to>
     <xdr:graphicFrame macro="">
@@ -6785,7 +6865,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="B3:M64"/>
+  <dimension ref="B3:M70"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="21.85546875" bestFit="1" customWidth="1"/>
@@ -6843,10 +6923,10 @@
         <v>11</v>
       </c>
       <c r="E5" s="4">
-        <v>10</v>
-      </c>
-      <c r="F5" s="17">
-        <v>1449</v>
+        <v>5</v>
+      </c>
+      <c r="F5" s="27">
+        <v>1096</v>
       </c>
       <c r="I5" s="9" t="s">
         <v>1</v>
@@ -6858,10 +6938,10 @@
         <v>11</v>
       </c>
       <c r="L5" s="4">
-        <v>10</v>
-      </c>
-      <c r="M5" s="17">
-        <v>1574</v>
+        <v>5</v>
+      </c>
+      <c r="M5" s="27">
+        <v>1410</v>
       </c>
     </row>
     <row r="6" spans="2:13" x14ac:dyDescent="0.25">
@@ -6875,10 +6955,10 @@
         <v>11</v>
       </c>
       <c r="E6" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F6" s="17">
-        <v>1802</v>
+        <v>1449</v>
       </c>
       <c r="I6" s="9" t="s">
         <v>1</v>
@@ -6890,10 +6970,10 @@
         <v>11</v>
       </c>
       <c r="L6" s="4">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="M6" s="17">
-        <v>1738</v>
+        <v>1574</v>
       </c>
     </row>
     <row r="7" spans="2:13" x14ac:dyDescent="0.25">
@@ -6907,10 +6987,10 @@
         <v>11</v>
       </c>
       <c r="E7" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="F7" s="17">
-        <v>2155</v>
+        <v>1802</v>
       </c>
       <c r="I7" s="9" t="s">
         <v>1</v>
@@ -6922,10 +7002,10 @@
         <v>11</v>
       </c>
       <c r="L7" s="4">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="M7" s="17">
-        <v>1900</v>
+        <v>1738</v>
       </c>
     </row>
     <row r="8" spans="2:13" x14ac:dyDescent="0.25">
@@ -6939,10 +7019,10 @@
         <v>11</v>
       </c>
       <c r="E8" s="4">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="F8" s="17">
-        <v>2508</v>
+        <v>2155</v>
       </c>
       <c r="I8" s="9" t="s">
         <v>1</v>
@@ -6954,10 +7034,10 @@
         <v>11</v>
       </c>
       <c r="L8" s="4">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="M8" s="17">
-        <v>2066</v>
+        <v>1900</v>
       </c>
     </row>
     <row r="9" spans="2:13" x14ac:dyDescent="0.25">
@@ -6971,10 +7051,10 @@
         <v>11</v>
       </c>
       <c r="E9" s="4">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="F9" s="17">
-        <v>2861</v>
+        <v>2508</v>
       </c>
       <c r="I9" s="9" t="s">
         <v>1</v>
@@ -6986,55 +7066,55 @@
         <v>11</v>
       </c>
       <c r="L9" s="4">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="M9" s="17">
-        <v>2230</v>
+        <v>2066</v>
       </c>
     </row>
     <row r="10" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B10" s="10"/>
-      <c r="C10" s="1"/>
-      <c r="D10" s="1"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="18"/>
-      <c r="I10" s="10"/>
-      <c r="J10" s="1"/>
-      <c r="K10" s="1"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="18"/>
+      <c r="B10" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="C10" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E10" s="4">
+        <v>30</v>
+      </c>
+      <c r="F10" s="17">
+        <v>2861</v>
+      </c>
+      <c r="I10" s="9" t="s">
+        <v>1</v>
+      </c>
+      <c r="J10" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K10" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L10" s="4">
+        <v>30</v>
+      </c>
+      <c r="M10" s="17">
+        <v>2230</v>
+      </c>
     </row>
     <row r="11" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B11" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E11" s="6">
-        <v>10</v>
-      </c>
-      <c r="F11" s="19">
-        <v>1521</v>
-      </c>
-      <c r="I11" s="11" t="s">
-        <v>3</v>
-      </c>
-      <c r="J11" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L11" s="6">
-        <v>10</v>
-      </c>
-      <c r="M11" s="19">
-        <v>1436</v>
-      </c>
+      <c r="B11" s="10"/>
+      <c r="C11" s="1"/>
+      <c r="D11" s="1"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="18"/>
+      <c r="I11" s="10"/>
+      <c r="J11" s="1"/>
+      <c r="K11" s="1"/>
+      <c r="L11" s="2"/>
+      <c r="M11" s="18"/>
     </row>
     <row r="12" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B12" s="11" t="s">
@@ -7047,10 +7127,10 @@
         <v>11</v>
       </c>
       <c r="E12" s="6">
-        <v>15</v>
-      </c>
-      <c r="F12" s="19">
-        <v>1891</v>
+        <v>5</v>
+      </c>
+      <c r="F12" s="18">
+        <v>1156</v>
       </c>
       <c r="I12" s="11" t="s">
         <v>3</v>
@@ -7062,10 +7142,10 @@
         <v>11</v>
       </c>
       <c r="L12" s="6">
-        <v>15</v>
-      </c>
-      <c r="M12" s="19">
-        <v>1610</v>
+        <v>5</v>
+      </c>
+      <c r="M12" s="18">
+        <v>1263</v>
       </c>
     </row>
     <row r="13" spans="2:13" x14ac:dyDescent="0.25">
@@ -7079,10 +7159,10 @@
         <v>11</v>
       </c>
       <c r="E13" s="6">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="F13" s="19">
-        <v>2256</v>
+        <v>1521</v>
       </c>
       <c r="I13" s="11" t="s">
         <v>3</v>
@@ -7094,10 +7174,10 @@
         <v>11</v>
       </c>
       <c r="L13" s="6">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="M13" s="19">
-        <v>1784</v>
+        <v>1436</v>
       </c>
     </row>
     <row r="14" spans="2:13" x14ac:dyDescent="0.25">
@@ -7111,10 +7191,10 @@
         <v>11</v>
       </c>
       <c r="E14" s="6">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="F14" s="19">
-        <v>2620</v>
+        <v>1891</v>
       </c>
       <c r="I14" s="11" t="s">
         <v>3</v>
@@ -7126,10 +7206,10 @@
         <v>11</v>
       </c>
       <c r="L14" s="6">
-        <v>25</v>
+        <v>15</v>
       </c>
       <c r="M14" s="19">
-        <v>1955</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="15" spans="2:13" x14ac:dyDescent="0.25">
@@ -7143,10 +7223,10 @@
         <v>11</v>
       </c>
       <c r="E15" s="6">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="F15" s="19">
-        <v>2991</v>
+        <v>2256</v>
       </c>
       <c r="I15" s="11" t="s">
         <v>3</v>
@@ -7158,87 +7238,87 @@
         <v>11</v>
       </c>
       <c r="L15" s="6">
-        <v>30</v>
+        <v>20</v>
       </c>
       <c r="M15" s="19">
-        <v>2132</v>
+        <v>1784</v>
       </c>
     </row>
     <row r="16" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B16" s="10"/>
-      <c r="C16" s="1"/>
-      <c r="D16" s="1"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="18"/>
-      <c r="I16" s="10"/>
-      <c r="J16" s="1"/>
-      <c r="K16" s="1"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="18"/>
+      <c r="B16" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C16" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E16" s="6">
+        <v>25</v>
+      </c>
+      <c r="F16" s="19">
+        <v>2620</v>
+      </c>
+      <c r="I16" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J16" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K16" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L16" s="6">
+        <v>25</v>
+      </c>
+      <c r="M16" s="19">
+        <v>1955</v>
+      </c>
     </row>
     <row r="17" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B17" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C17" s="3" t="s">
+      <c r="B17" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D17" s="3" t="s">
+      <c r="D17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E17" s="4">
-        <v>10</v>
-      </c>
-      <c r="F17" s="17">
-        <v>527</v>
-      </c>
-      <c r="I17" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J17" s="3" t="s">
+      <c r="E17" s="6">
+        <v>30</v>
+      </c>
+      <c r="F17" s="19">
+        <v>2991</v>
+      </c>
+      <c r="I17" s="11" t="s">
+        <v>3</v>
+      </c>
+      <c r="J17" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K17" s="3" t="s">
+      <c r="K17" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L17" s="4">
-        <v>10</v>
-      </c>
-      <c r="M17" s="17">
-        <v>540</v>
+      <c r="L17" s="6">
+        <v>30</v>
+      </c>
+      <c r="M17" s="19">
+        <v>2132</v>
       </c>
     </row>
     <row r="18" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B18" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="C18" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E18" s="4">
-        <v>15</v>
-      </c>
-      <c r="F18" s="17">
-        <v>698</v>
-      </c>
-      <c r="I18" s="9" t="s">
-        <v>4</v>
-      </c>
-      <c r="J18" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K18" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="L18" s="4">
-        <v>15</v>
-      </c>
-      <c r="M18" s="17">
-        <v>620</v>
-      </c>
+      <c r="B18" s="10"/>
+      <c r="C18" s="1"/>
+      <c r="D18" s="1"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="18"/>
+      <c r="I18" s="10"/>
+      <c r="J18" s="1"/>
+      <c r="K18" s="1"/>
+      <c r="L18" s="2"/>
+      <c r="M18" s="18"/>
     </row>
     <row r="19" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B19" s="9" t="s">
@@ -7251,10 +7331,10 @@
         <v>11</v>
       </c>
       <c r="E19" s="4">
-        <v>20</v>
-      </c>
-      <c r="F19" s="17">
-        <v>863</v>
+        <v>5</v>
+      </c>
+      <c r="F19" s="18">
+        <v>362</v>
       </c>
       <c r="I19" s="9" t="s">
         <v>4</v>
@@ -7266,10 +7346,10 @@
         <v>11</v>
       </c>
       <c r="L19" s="4">
-        <v>20</v>
-      </c>
-      <c r="M19" s="17">
-        <v>700</v>
+        <v>5</v>
+      </c>
+      <c r="M19" s="18">
+        <v>460</v>
       </c>
     </row>
     <row r="20" spans="2:13" x14ac:dyDescent="0.25">
@@ -7283,10 +7363,10 @@
         <v>11</v>
       </c>
       <c r="E20" s="4">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="F20" s="17">
-        <v>1028</v>
+        <v>527</v>
       </c>
       <c r="I20" s="9" t="s">
         <v>4</v>
@@ -7298,10 +7378,10 @@
         <v>11</v>
       </c>
       <c r="L20" s="4">
-        <v>25</v>
+        <v>10</v>
       </c>
       <c r="M20" s="17">
-        <v>777</v>
+        <v>540</v>
       </c>
     </row>
     <row r="21" spans="2:13" x14ac:dyDescent="0.25">
@@ -7315,10 +7395,10 @@
         <v>11</v>
       </c>
       <c r="E21" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="F21" s="17">
-        <v>1199</v>
+        <v>698</v>
       </c>
       <c r="I21" s="9" t="s">
         <v>4</v>
@@ -7330,119 +7410,119 @@
         <v>11</v>
       </c>
       <c r="L21" s="4">
-        <v>30</v>
+        <v>15</v>
       </c>
       <c r="M21" s="17">
-        <v>860</v>
+        <v>620</v>
       </c>
     </row>
     <row r="22" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B22" s="10"/>
-      <c r="C22" s="1"/>
-      <c r="D22" s="1"/>
-      <c r="E22" s="2"/>
-      <c r="F22" s="18"/>
-      <c r="I22" s="10"/>
-      <c r="J22" s="1"/>
-      <c r="K22" s="1"/>
-      <c r="L22" s="2"/>
-      <c r="M22" s="18"/>
+      <c r="B22" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E22" s="4">
+        <v>20</v>
+      </c>
+      <c r="F22" s="17">
+        <v>863</v>
+      </c>
+      <c r="I22" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J22" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K22" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L22" s="4">
+        <v>20</v>
+      </c>
+      <c r="M22" s="17">
+        <v>700</v>
+      </c>
     </row>
     <row r="23" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B23" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C23" s="5" t="s">
+      <c r="B23" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C23" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D23" s="5" t="s">
+      <c r="D23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E23" s="6">
-        <v>10</v>
-      </c>
-      <c r="F23" s="19">
-        <v>260</v>
-      </c>
-      <c r="I23" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J23" s="5" t="s">
+      <c r="E23" s="4">
+        <v>25</v>
+      </c>
+      <c r="F23" s="17">
+        <v>1028</v>
+      </c>
+      <c r="I23" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J23" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K23" s="5" t="s">
+      <c r="K23" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L23" s="6">
-        <v>10</v>
-      </c>
-      <c r="M23" s="19">
-        <v>270</v>
+      <c r="L23" s="4">
+        <v>25</v>
+      </c>
+      <c r="M23" s="17">
+        <v>777</v>
       </c>
     </row>
     <row r="24" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B24" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C24" s="5" t="s">
+      <c r="B24" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="C24" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D24" s="5" t="s">
+      <c r="D24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E24" s="6">
-        <v>15</v>
-      </c>
-      <c r="F24" s="19">
-        <v>366</v>
-      </c>
-      <c r="I24" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J24" s="5" t="s">
+      <c r="E24" s="4">
+        <v>30</v>
+      </c>
+      <c r="F24" s="17">
+        <v>1199</v>
+      </c>
+      <c r="I24" s="9" t="s">
+        <v>4</v>
+      </c>
+      <c r="J24" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K24" s="5" t="s">
+      <c r="K24" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L24" s="6">
-        <v>15</v>
-      </c>
-      <c r="M24" s="19">
-        <v>323</v>
+      <c r="L24" s="4">
+        <v>30</v>
+      </c>
+      <c r="M24" s="17">
+        <v>860</v>
       </c>
     </row>
     <row r="25" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B25" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="C25" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="D25" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="E25" s="6">
-        <v>20</v>
-      </c>
-      <c r="F25" s="19">
-        <v>467</v>
-      </c>
-      <c r="I25" s="11" t="s">
-        <v>5</v>
-      </c>
-      <c r="J25" s="5" t="s">
-        <v>13</v>
-      </c>
-      <c r="K25" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="L25" s="6">
-        <v>20</v>
-      </c>
-      <c r="M25" s="19">
-        <v>375</v>
-      </c>
+      <c r="B25" s="10"/>
+      <c r="C25" s="1"/>
+      <c r="D25" s="1"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="18"/>
+      <c r="I25" s="10"/>
+      <c r="J25" s="1"/>
+      <c r="K25" s="1"/>
+      <c r="L25" s="2"/>
+      <c r="M25" s="18"/>
     </row>
     <row r="26" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B26" s="11" t="s">
@@ -7455,10 +7535,10 @@
         <v>11</v>
       </c>
       <c r="E26" s="6">
-        <v>25</v>
-      </c>
-      <c r="F26" s="19">
-        <v>568</v>
+        <v>5</v>
+      </c>
+      <c r="F26" s="18">
+        <v>159</v>
       </c>
       <c r="I26" s="11" t="s">
         <v>5</v>
@@ -7470,10 +7550,10 @@
         <v>11</v>
       </c>
       <c r="L26" s="6">
-        <v>25</v>
-      </c>
-      <c r="M26" s="19">
-        <v>428</v>
+        <v>5</v>
+      </c>
+      <c r="M26" s="18">
+        <v>217</v>
       </c>
     </row>
     <row r="27" spans="2:13" x14ac:dyDescent="0.25">
@@ -7487,10 +7567,10 @@
         <v>11</v>
       </c>
       <c r="E27" s="6">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="F27" s="19">
-        <v>674</v>
+        <v>260</v>
       </c>
       <c r="I27" s="11" t="s">
         <v>5</v>
@@ -7502,151 +7582,151 @@
         <v>11</v>
       </c>
       <c r="L27" s="6">
-        <v>30</v>
+        <v>10</v>
       </c>
       <c r="M27" s="19">
-        <v>481</v>
+        <v>270</v>
       </c>
     </row>
     <row r="28" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B28" s="10"/>
-      <c r="C28" s="1"/>
-      <c r="D28" s="1"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="18"/>
-      <c r="I28" s="10"/>
-      <c r="J28" s="1"/>
-      <c r="K28" s="1"/>
-      <c r="L28" s="2"/>
-      <c r="M28" s="18"/>
+      <c r="B28" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E28" s="6">
+        <v>15</v>
+      </c>
+      <c r="F28" s="19">
+        <v>366</v>
+      </c>
+      <c r="I28" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J28" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K28" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L28" s="6">
+        <v>15</v>
+      </c>
+      <c r="M28" s="19">
+        <v>323</v>
+      </c>
     </row>
     <row r="29" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B29" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C29" s="3" t="s">
+      <c r="B29" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D29" s="3" t="s">
+      <c r="D29" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E29" s="4">
-        <v>10</v>
-      </c>
-      <c r="F29" s="17">
-        <v>1446</v>
-      </c>
-      <c r="I29" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J29" s="3" t="s">
+      <c r="E29" s="6">
+        <v>20</v>
+      </c>
+      <c r="F29" s="19">
+        <v>467</v>
+      </c>
+      <c r="I29" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J29" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K29" s="3" t="s">
+      <c r="K29" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L29" s="4">
-        <v>10</v>
-      </c>
-      <c r="M29" s="17">
-        <v>1384</v>
+      <c r="L29" s="6">
+        <v>20</v>
+      </c>
+      <c r="M29" s="19">
+        <v>375</v>
       </c>
     </row>
     <row r="30" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B30" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C30" s="3" t="s">
+      <c r="B30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D30" s="3" t="s">
+      <c r="D30" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E30" s="4">
-        <v>15</v>
-      </c>
-      <c r="F30" s="17">
-        <v>1798</v>
-      </c>
-      <c r="I30" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J30" s="3" t="s">
+      <c r="E30" s="6">
+        <v>25</v>
+      </c>
+      <c r="F30" s="19">
+        <v>568</v>
+      </c>
+      <c r="I30" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J30" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K30" s="3" t="s">
+      <c r="K30" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L30" s="4">
-        <v>15</v>
-      </c>
-      <c r="M30" s="17">
-        <v>1549</v>
+      <c r="L30" s="6">
+        <v>25</v>
+      </c>
+      <c r="M30" s="19">
+        <v>428</v>
       </c>
     </row>
     <row r="31" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B31" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C31" s="3" t="s">
+      <c r="B31" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="C31" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D31" s="3" t="s">
+      <c r="D31" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E31" s="4">
-        <v>20</v>
-      </c>
-      <c r="F31" s="17">
-        <v>2150</v>
-      </c>
-      <c r="I31" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J31" s="3" t="s">
+      <c r="E31" s="6">
+        <v>30</v>
+      </c>
+      <c r="F31" s="19">
+        <v>674</v>
+      </c>
+      <c r="I31" s="11" t="s">
+        <v>5</v>
+      </c>
+      <c r="J31" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K31" s="3" t="s">
+      <c r="K31" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L31" s="4">
-        <v>20</v>
-      </c>
-      <c r="M31" s="17">
-        <v>1719</v>
+      <c r="L31" s="6">
+        <v>30</v>
+      </c>
+      <c r="M31" s="19">
+        <v>481</v>
       </c>
     </row>
     <row r="32" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B32" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="E32" s="4">
-        <v>25</v>
-      </c>
-      <c r="F32" s="17">
-        <v>2501</v>
-      </c>
-      <c r="I32" s="9" t="s">
-        <v>6</v>
-      </c>
-      <c r="J32" s="3" t="s">
-        <v>13</v>
-      </c>
-      <c r="K32" s="3" t="s">
-        <v>11</v>
-      </c>
-      <c r="L32" s="4">
-        <v>25</v>
-      </c>
-      <c r="M32" s="17">
-        <v>1883</v>
-      </c>
+      <c r="B32" s="10"/>
+      <c r="C32" s="1"/>
+      <c r="D32" s="1"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="18"/>
+      <c r="I32" s="10"/>
+      <c r="J32" s="1"/>
+      <c r="K32" s="1"/>
+      <c r="L32" s="2"/>
+      <c r="M32" s="18"/>
     </row>
     <row r="33" spans="2:13" x14ac:dyDescent="0.25">
       <c r="B33" s="9" t="s">
@@ -7659,10 +7739,10 @@
         <v>11</v>
       </c>
       <c r="E33" s="4">
-        <v>30</v>
-      </c>
-      <c r="F33" s="17">
-        <v>2852</v>
+        <v>5</v>
+      </c>
+      <c r="F33" s="18">
+        <v>1093</v>
       </c>
       <c r="I33" s="9" t="s">
         <v>6</v>
@@ -7674,308 +7754,414 @@
         <v>11</v>
       </c>
       <c r="L33" s="4">
-        <v>30</v>
-      </c>
-      <c r="M33" s="17">
-        <v>2053</v>
+        <v>5</v>
+      </c>
+      <c r="M33" s="18">
+        <v>1215</v>
       </c>
     </row>
     <row r="34" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B34" s="10"/>
-      <c r="C34" s="1"/>
-      <c r="D34" s="1"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="18"/>
-      <c r="I34" s="10"/>
-      <c r="J34" s="1"/>
-      <c r="K34" s="1"/>
-      <c r="L34" s="2"/>
-      <c r="M34" s="18"/>
+      <c r="B34" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E34" s="4">
+        <v>10</v>
+      </c>
+      <c r="F34" s="17">
+        <v>1446</v>
+      </c>
+      <c r="I34" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J34" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K34" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L34" s="4">
+        <v>10</v>
+      </c>
+      <c r="M34" s="17">
+        <v>1384</v>
+      </c>
     </row>
     <row r="35" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B35" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C35" s="5" t="s">
+      <c r="B35" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C35" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D35" s="5" t="s">
+      <c r="D35" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E35" s="6">
-        <v>10</v>
-      </c>
-      <c r="F35" s="19">
-        <v>675</v>
-      </c>
-      <c r="I35" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="J35" s="5" t="s">
+      <c r="E35" s="4">
+        <v>15</v>
+      </c>
+      <c r="F35" s="17">
+        <v>1798</v>
+      </c>
+      <c r="I35" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J35" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K35" s="5" t="s">
+      <c r="K35" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L35" s="6">
-        <v>10</v>
-      </c>
-      <c r="M35" s="19">
-        <v>659</v>
+      <c r="L35" s="4">
+        <v>15</v>
+      </c>
+      <c r="M35" s="17">
+        <v>1549</v>
       </c>
     </row>
     <row r="36" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B36" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C36" s="5" t="s">
+      <c r="B36" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C36" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D36" s="5" t="s">
+      <c r="D36" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E36" s="6">
-        <v>15</v>
-      </c>
-      <c r="F36" s="19">
-        <v>870</v>
-      </c>
-      <c r="I36" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="J36" s="5" t="s">
+      <c r="E36" s="4">
+        <v>20</v>
+      </c>
+      <c r="F36" s="17">
+        <v>2150</v>
+      </c>
+      <c r="I36" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J36" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K36" s="5" t="s">
+      <c r="K36" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L36" s="6">
-        <v>15</v>
-      </c>
-      <c r="M36" s="19">
-        <v>747</v>
+      <c r="L36" s="4">
+        <v>20</v>
+      </c>
+      <c r="M36" s="17">
+        <v>1719</v>
       </c>
     </row>
     <row r="37" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B37" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="C37" s="5" t="s">
+      <c r="B37" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C37" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="D37" s="5" t="s">
+      <c r="D37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="E37" s="6">
-        <v>20</v>
-      </c>
-      <c r="F37" s="19">
-        <v>1067</v>
-      </c>
-      <c r="I37" s="11" t="s">
-        <v>7</v>
-      </c>
-      <c r="J37" s="5" t="s">
+      <c r="E37" s="4">
+        <v>25</v>
+      </c>
+      <c r="F37" s="17">
+        <v>2501</v>
+      </c>
+      <c r="I37" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J37" s="3" t="s">
         <v>13</v>
       </c>
-      <c r="K37" s="5" t="s">
+      <c r="K37" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="L37" s="6">
-        <v>20</v>
-      </c>
-      <c r="M37" s="19">
-        <v>840</v>
+      <c r="L37" s="4">
+        <v>25</v>
+      </c>
+      <c r="M37" s="17">
+        <v>1883</v>
       </c>
     </row>
     <row r="38" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B38" s="11" t="s">
+      <c r="B38" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>9</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="E38" s="4">
+        <v>30</v>
+      </c>
+      <c r="F38" s="17">
+        <v>2852</v>
+      </c>
+      <c r="I38" s="9" t="s">
+        <v>6</v>
+      </c>
+      <c r="J38" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K38" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="L38" s="4">
+        <v>30</v>
+      </c>
+      <c r="M38" s="17">
+        <v>2053</v>
+      </c>
+    </row>
+    <row r="39" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B39" s="10"/>
+      <c r="C39" s="1"/>
+      <c r="D39" s="1"/>
+      <c r="E39" s="2"/>
+      <c r="F39" s="18"/>
+      <c r="I39" s="10"/>
+      <c r="J39" s="1"/>
+      <c r="K39" s="1"/>
+      <c r="L39" s="2"/>
+      <c r="M39" s="18"/>
+    </row>
+    <row r="40" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B40" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C38" s="5" t="s">
+      <c r="C40" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D38" s="5" t="s">
+      <c r="D40" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E38" s="6">
-        <v>25</v>
-      </c>
-      <c r="F38" s="19">
-        <v>1264</v>
-      </c>
-      <c r="I38" s="11" t="s">
+      <c r="E40" s="6">
+        <v>5</v>
+      </c>
+      <c r="F40" s="18">
+        <v>474</v>
+      </c>
+      <c r="I40" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J38" s="5" t="s">
+      <c r="J40" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K38" s="5" t="s">
+      <c r="K40" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L38" s="6">
-        <v>25</v>
-      </c>
-      <c r="M38" s="19">
-        <v>927</v>
+      <c r="L40" s="6">
+        <v>5</v>
+      </c>
+      <c r="M40" s="18">
+        <v>572</v>
       </c>
     </row>
-    <row r="39" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="B39" s="12" t="s">
+    <row r="41" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B41" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="C39" s="7" t="s">
+      <c r="C41" s="5" t="s">
         <v>9</v>
       </c>
-      <c r="D39" s="7" t="s">
+      <c r="D41" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E39" s="8">
-        <v>30</v>
-      </c>
-      <c r="F39" s="20">
-        <v>1462</v>
-      </c>
-      <c r="I39" s="12" t="s">
+      <c r="E41" s="6">
+        <v>10</v>
+      </c>
+      <c r="F41" s="19">
+        <v>675</v>
+      </c>
+      <c r="I41" s="11" t="s">
         <v>7</v>
       </c>
-      <c r="J39" s="7" t="s">
+      <c r="J41" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="K39" s="7" t="s">
+      <c r="K41" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="L39" s="8">
-        <v>30</v>
-      </c>
-      <c r="M39" s="20">
-        <v>1015</v>
+      <c r="L41" s="6">
+        <v>10</v>
+      </c>
+      <c r="M41" s="19">
+        <v>659</v>
       </c>
     </row>
     <row r="42" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B42" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C42" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="D42" s="21" t="s">
+      <c r="B42" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C42" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E42" s="6">
         <v>15</v>
       </c>
-      <c r="I42" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="J42" s="21" t="s">
-        <v>14</v>
-      </c>
-      <c r="K42" s="21" t="s">
+      <c r="F42" s="19">
+        <v>870</v>
+      </c>
+      <c r="I42" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J42" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K42" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L42" s="6">
         <v>15</v>
       </c>
+      <c r="M42" s="19">
+        <v>747</v>
+      </c>
     </row>
-    <row r="43" spans="2:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="B43" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C43" t="s">
-        <v>16</v>
-      </c>
-      <c r="D43" t="s">
-        <v>17</v>
-      </c>
-      <c r="I43" s="25" t="s">
-        <v>50</v>
-      </c>
-      <c r="J43" t="s">
-        <v>16</v>
-      </c>
-      <c r="K43" t="s">
-        <v>17</v>
+    <row r="43" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B43" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E43" s="6">
+        <v>20</v>
+      </c>
+      <c r="F43" s="19">
+        <v>1067</v>
+      </c>
+      <c r="I43" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J43" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K43" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L43" s="6">
+        <v>20</v>
+      </c>
+      <c r="M43" s="19">
+        <v>840</v>
       </c>
     </row>
-    <row r="44" spans="2:13" ht="30" x14ac:dyDescent="0.25">
-      <c r="B44" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="C44" t="s">
-        <v>18</v>
-      </c>
-      <c r="D44" t="s">
-        <v>19</v>
-      </c>
-      <c r="I44" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="J44" t="s">
-        <v>18</v>
-      </c>
-      <c r="K44" t="s">
-        <v>19</v>
+    <row r="44" spans="2:13" x14ac:dyDescent="0.25">
+      <c r="B44" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="C44" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="D44" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="E44" s="6">
+        <v>25</v>
+      </c>
+      <c r="F44" s="19">
+        <v>1264</v>
+      </c>
+      <c r="I44" s="11" t="s">
+        <v>7</v>
+      </c>
+      <c r="J44" s="5" t="s">
+        <v>13</v>
+      </c>
+      <c r="K44" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="L44" s="6">
+        <v>25</v>
+      </c>
+      <c r="M44" s="19">
+        <v>927</v>
       </c>
     </row>
-    <row r="45" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B45" s="21" t="s">
-        <v>36</v>
-      </c>
-      <c r="C45" t="s">
-        <v>20</v>
-      </c>
-      <c r="D45" t="s">
-        <v>21</v>
-      </c>
-      <c r="I45" s="26" t="s">
-        <v>36</v>
-      </c>
-      <c r="J45" t="s">
-        <v>20</v>
-      </c>
-      <c r="K45" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="46" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="I46" s="24"/>
-    </row>
-    <row r="47" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="B47" t="s">
-        <v>35</v>
-      </c>
-      <c r="C47" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="D47" t="s">
-        <v>23</v>
-      </c>
-      <c r="I47" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="J47" s="22" t="s">
-        <v>22</v>
-      </c>
-      <c r="K47" t="s">
-        <v>39</v>
+    <row r="45" spans="2:13" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="B45" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C45" s="7" t="s">
+        <v>9</v>
+      </c>
+      <c r="D45" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="E45" s="8">
+        <v>30</v>
+      </c>
+      <c r="F45" s="20">
+        <v>1462</v>
+      </c>
+      <c r="I45" s="12" t="s">
+        <v>7</v>
+      </c>
+      <c r="J45" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="K45" s="7" t="s">
+        <v>11</v>
+      </c>
+      <c r="L45" s="8">
+        <v>30</v>
+      </c>
+      <c r="M45" s="20">
+        <v>1015</v>
       </c>
     </row>
     <row r="48" spans="2:13" x14ac:dyDescent="0.25">
-      <c r="I48" s="24"/>
+      <c r="B48" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C48" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="D48" s="21" t="s">
+        <v>15</v>
+      </c>
+      <c r="I48" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J48" s="21" t="s">
+        <v>14</v>
+      </c>
+      <c r="K48" s="21" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="49" spans="2:11" ht="30" x14ac:dyDescent="0.25">
       <c r="B49" s="25" t="s">
         <v>37</v>
       </c>
       <c r="C49" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="D49" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="I49" s="25" t="s">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="J49" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="K49" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
     </row>
     <row r="50" spans="2:11" ht="30" x14ac:dyDescent="0.25">
@@ -7983,165 +8169,251 @@
         <v>37</v>
       </c>
       <c r="C50" t="s">
-        <v>26</v>
-      </c>
-      <c r="D50" s="23">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="D50" t="s">
+        <v>19</v>
       </c>
       <c r="I50" s="25" t="s">
         <v>37</v>
       </c>
       <c r="J50" t="s">
-        <v>26</v>
-      </c>
-      <c r="K50" s="23">
-        <v>1</v>
+        <v>18</v>
+      </c>
+      <c r="K50" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="51" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I51" s="24"/>
+      <c r="B51" s="21" t="s">
+        <v>36</v>
+      </c>
+      <c r="C51" t="s">
+        <v>20</v>
+      </c>
+      <c r="D51" t="s">
+        <v>21</v>
+      </c>
+      <c r="I51" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J51" t="s">
+        <v>20</v>
+      </c>
+      <c r="K51" t="s">
+        <v>38</v>
+      </c>
     </row>
     <row r="52" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B52" t="s">
-        <v>35</v>
-      </c>
-      <c r="C52" t="s">
-        <v>27</v>
-      </c>
-      <c r="D52" t="s">
-        <v>28</v>
-      </c>
-      <c r="I52" s="24" t="s">
-        <v>35</v>
-      </c>
-      <c r="J52" t="s">
-        <v>27</v>
-      </c>
-      <c r="K52" t="s">
-        <v>40</v>
-      </c>
+      <c r="I52" s="24"/>
     </row>
     <row r="53" spans="2:11" x14ac:dyDescent="0.25">
       <c r="B53" t="s">
         <v>35</v>
       </c>
-      <c r="C53" t="s">
-        <v>29</v>
+      <c r="C53" s="22" t="s">
+        <v>22</v>
       </c>
       <c r="D53" t="s">
-        <v>30</v>
+        <v>23</v>
       </c>
       <c r="I53" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="J53" t="s">
-        <v>29</v>
+      <c r="J53" s="22" t="s">
+        <v>22</v>
       </c>
       <c r="K53" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="54" spans="2:11" x14ac:dyDescent="0.25">
       <c r="I54" s="24"/>
     </row>
-    <row r="55" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B55" t="s">
-        <v>36</v>
+    <row r="55" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B55" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C55" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="D55" t="s">
-        <v>32</v>
-      </c>
-      <c r="I55" s="24" t="s">
-        <v>36</v>
+        <v>25</v>
+      </c>
+      <c r="I55" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="J55" t="s">
-        <v>31</v>
+        <v>24</v>
       </c>
       <c r="K55" t="s">
-        <v>32</v>
+        <v>25</v>
       </c>
     </row>
-    <row r="56" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="B56" t="s">
-        <v>36</v>
+    <row r="56" spans="2:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="B56" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="C56" t="s">
-        <v>33</v>
-      </c>
-      <c r="D56" t="s">
-        <v>34</v>
-      </c>
-      <c r="I56" s="24" t="s">
-        <v>36</v>
+        <v>26</v>
+      </c>
+      <c r="D56" s="23">
+        <v>1</v>
+      </c>
+      <c r="I56" s="25" t="s">
+        <v>37</v>
       </c>
       <c r="J56" t="s">
-        <v>33</v>
-      </c>
-      <c r="K56" t="s">
-        <v>34</v>
+        <v>26</v>
+      </c>
+      <c r="K56" s="23">
+        <v>1</v>
       </c>
     </row>
     <row r="57" spans="2:11" x14ac:dyDescent="0.25">
       <c r="I57" s="24"/>
     </row>
     <row r="58" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I58" s="24"/>
+      <c r="B58" t="s">
+        <v>35</v>
+      </c>
+      <c r="C58" t="s">
+        <v>27</v>
+      </c>
+      <c r="D58" t="s">
+        <v>28</v>
+      </c>
+      <c r="I58" s="24" t="s">
+        <v>35</v>
+      </c>
+      <c r="J58" t="s">
+        <v>27</v>
+      </c>
+      <c r="K58" t="s">
+        <v>40</v>
+      </c>
     </row>
-    <row r="59" spans="2:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="I59" s="25" t="s">
-        <v>37</v>
+    <row r="59" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B59" t="s">
+        <v>35</v>
+      </c>
+      <c r="C59" t="s">
+        <v>29</v>
+      </c>
+      <c r="D59" t="s">
+        <v>30</v>
+      </c>
+      <c r="I59" s="24" t="s">
+        <v>35</v>
       </c>
       <c r="J59" t="s">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="K59" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
-    <row r="60" spans="2:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="I60" s="25" t="s">
-        <v>37</v>
-      </c>
-      <c r="J60" t="s">
-        <v>44</v>
-      </c>
-      <c r="K60" t="s">
-        <v>45</v>
-      </c>
+    <row r="60" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I60" s="24"/>
     </row>
-    <row r="61" spans="2:11" ht="30" x14ac:dyDescent="0.25">
-      <c r="I61" s="25" t="s">
-        <v>37</v>
+    <row r="61" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="B61" t="s">
+        <v>36</v>
+      </c>
+      <c r="C61" t="s">
+        <v>31</v>
+      </c>
+      <c r="D61" t="s">
+        <v>32</v>
+      </c>
+      <c r="I61" s="24" t="s">
+        <v>36</v>
       </c>
       <c r="J61" t="s">
-        <v>46</v>
+        <v>31</v>
       </c>
       <c r="K61" t="s">
-        <v>47</v>
+        <v>32</v>
       </c>
     </row>
     <row r="62" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I62" s="26" t="s">
+      <c r="B62" t="s">
         <v>36</v>
       </c>
+      <c r="C62" t="s">
+        <v>33</v>
+      </c>
+      <c r="D62" t="s">
+        <v>34</v>
+      </c>
+      <c r="I62" s="24" t="s">
+        <v>36</v>
+      </c>
       <c r="J62" t="s">
-        <v>20</v>
+        <v>33</v>
       </c>
       <c r="K62" t="s">
-        <v>38</v>
-      </c>
+        <v>34</v>
+      </c>
+    </row>
+    <row r="63" spans="2:11" x14ac:dyDescent="0.25">
+      <c r="I63" s="24"/>
     </row>
     <row r="64" spans="2:11" x14ac:dyDescent="0.25">
-      <c r="I64" s="24" t="s">
+      <c r="I64" s="24"/>
+    </row>
+    <row r="65" spans="9:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="I65" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="J65" t="s">
+        <v>42</v>
+      </c>
+      <c r="K65" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="66" spans="9:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="I66" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="J66" t="s">
+        <v>44</v>
+      </c>
+      <c r="K66" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="67" spans="9:11" ht="30" x14ac:dyDescent="0.25">
+      <c r="I67" s="25" t="s">
+        <v>37</v>
+      </c>
+      <c r="J67" t="s">
+        <v>46</v>
+      </c>
+      <c r="K67" t="s">
+        <v>47</v>
+      </c>
+    </row>
+    <row r="68" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I68" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="J68" t="s">
+        <v>20</v>
+      </c>
+      <c r="K68" t="s">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="70" spans="9:11" x14ac:dyDescent="0.25">
+      <c r="I70" s="24" t="s">
         <v>35</v>
       </c>
-      <c r="J64" t="s">
+      <c r="J70" t="s">
         <v>48</v>
       </c>
-      <c r="K64" t="s">
+      <c r="K70" t="s">
         <v>49</v>
       </c>
     </row>

</xml_diff>